<commit_message>
Accept multiple spaces before year
</commit_message>
<xml_diff>
--- a/tests/VAGTSKEMA MARTS 2025 (002).xlsx
+++ b/tests/VAGTSKEMA MARTS 2025 (002).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meon\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vagtplan\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969B4516-F398-49A7-A27B-41B73DD677D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD77A90E-D80C-4E82-930D-570C9C885D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{8296F9AC-D2FD-40F5-8351-118E60B2EBF6}"/>
+    <workbookView xWindow="18420" yWindow="-16932" windowWidth="13188" windowHeight="17028" activeTab="1" xr2:uid="{8296F9AC-D2FD-40F5-8351-118E60B2EBF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark2" sheetId="2" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>ADI/PRO</t>
   </si>
   <si>
-    <t>BØRNE- OG UNGEAFDELINGEN MARTS 2025</t>
-  </si>
-  <si>
     <t>JN/LM</t>
   </si>
   <si>
@@ -511,6 +508,9 @@
   </si>
   <si>
     <t>ET SI BD JK BK AT JB</t>
+  </si>
+  <si>
+    <t>BØRNE- OG UNGEAFDELINGEN MARTS  2025</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1016,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB49BD5-47C1-481F-85CA-32D1C6275076}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -1027,34 +1027,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037BD9F7-5BE0-4720-B0E0-97FA7C61CA4C}">
   <dimension ref="A1:Q64"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" customWidth="1"/>
-    <col min="4" max="4" width="4.28515625" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" customWidth="1"/>
-    <col min="9" max="9" width="5.28515625" customWidth="1"/>
-    <col min="10" max="10" width="5.42578125" customWidth="1"/>
+    <col min="2" max="2" width="4.3046875" customWidth="1"/>
+    <col min="3" max="3" width="6.53515625" customWidth="1"/>
+    <col min="4" max="4" width="4.3046875" customWidth="1"/>
+    <col min="5" max="5" width="5.15234375" customWidth="1"/>
+    <col min="6" max="6" width="5.3828125" customWidth="1"/>
+    <col min="7" max="7" width="18.69140625" customWidth="1"/>
+    <col min="8" max="8" width="19.84375" customWidth="1"/>
+    <col min="9" max="9" width="5.3046875" customWidth="1"/>
+    <col min="10" max="10" width="5.3828125" customWidth="1"/>
     <col min="11" max="11" width="1" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="5.42578125" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" customWidth="1"/>
-    <col min="14" max="14" width="32.140625" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" customWidth="1"/>
-    <col min="16" max="16" width="8.7109375" customWidth="1"/>
+    <col min="12" max="12" width="5.3828125" customWidth="1"/>
+    <col min="13" max="13" width="9.3828125" customWidth="1"/>
+    <col min="14" max="14" width="32.15234375" customWidth="1"/>
+    <col min="15" max="15" width="10.84375" customWidth="1"/>
+    <col min="16" max="16" width="8.69140625" customWidth="1"/>
     <col min="17" max="17" width="8" customWidth="1"/>
-    <col min="18" max="18" width="7.28515625" customWidth="1"/>
+    <col min="18" max="18" width="7.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="19.75" x14ac:dyDescent="0.45">
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
       <c r="E1" s="27"/>
       <c r="F1" s="1" t="s">
-        <v>33</v>
+        <v>161</v>
       </c>
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
@@ -1064,14 +1064,14 @@
       <c r="L1" s="27"/>
       <c r="N1" s="20"/>
       <c r="O1" s="20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P1" s="6"/>
       <c r="Q1" s="48" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="12"/>
       <c r="B2" s="12" t="s">
         <v>0</v>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="Q2" s="47"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>9</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="30"/>
@@ -1142,11 +1142,11 @@
       <c r="M3" s="18"/>
       <c r="N3" s="18"/>
       <c r="O3" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P3" s="23"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>10</v>
       </c>
@@ -1154,12 +1154,12 @@
         <v>2</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" s="19"/>
       <c r="E4" s="30"/>
       <c r="F4" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G4" s="18"/>
       <c r="H4" s="18"/>
@@ -1170,13 +1170,13 @@
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P4" s="23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>5</v>
       </c>
@@ -1184,20 +1184,20 @@
         <v>3</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E5" s="24"/>
       <c r="F5" s="26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G5" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="26" t="s">
         <v>121</v>
-      </c>
-      <c r="H5" s="26" t="s">
-        <v>122</v>
       </c>
       <c r="I5" s="21"/>
       <c r="J5" s="21"/>
@@ -1207,17 +1207,17 @@
       </c>
       <c r="M5" s="16"/>
       <c r="N5" s="26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O5" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P5" s="21" t="s">
         <v>26</v>
       </c>
       <c r="Q5" s="45"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>11</v>
       </c>
@@ -1225,20 +1225,20 @@
         <v>4</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E6" s="40"/>
       <c r="F6" s="16" t="s">
         <v>26</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I6" s="21"/>
       <c r="J6" s="21"/>
@@ -1248,14 +1248,14 @@
         <v>28</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O6" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P6" s="21"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
         <v>6</v>
       </c>
@@ -1263,20 +1263,20 @@
         <v>5</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E7" s="24"/>
       <c r="F7" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I7" s="21" t="s">
         <v>27</v>
@@ -1288,15 +1288,15 @@
       </c>
       <c r="M7" s="16"/>
       <c r="N7" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O7" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P7" s="21"/>
       <c r="Q7" s="45"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
         <v>7</v>
       </c>
@@ -1304,37 +1304,37 @@
         <v>6</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I8" s="21"/>
       <c r="J8" s="21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K8" s="31"/>
       <c r="L8" s="21"/>
       <c r="M8" s="16"/>
       <c r="N8" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O8" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P8" s="21"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
         <v>8</v>
       </c>
@@ -1342,20 +1342,20 @@
         <v>7</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E9" s="31"/>
       <c r="F9" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G9" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="16" t="s">
         <v>125</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>126</v>
       </c>
       <c r="I9" s="21"/>
       <c r="J9" s="21"/>
@@ -1364,20 +1364,20 @@
         <v>27</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O9" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P9" s="21" t="s">
         <v>26</v>
       </c>
       <c r="Q9" s="46"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
         <v>9</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="30"/>
@@ -1401,11 +1401,11 @@
       <c r="M10" s="18"/>
       <c r="N10" s="18"/>
       <c r="O10" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P10" s="23"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="23" t="s">
         <v>10</v>
       </c>
@@ -1413,12 +1413,12 @@
         <v>9</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="30"/>
       <c r="F11" s="18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G11" s="18"/>
       <c r="H11" s="18"/>
@@ -1429,11 +1429,11 @@
       <c r="M11" s="18"/>
       <c r="N11" s="18"/>
       <c r="O11" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P11" s="23"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>5</v>
       </c>
@@ -1441,38 +1441,38 @@
         <v>10</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12" s="21"/>
       <c r="F12" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
       <c r="K12" s="31"/>
       <c r="L12" s="21"/>
       <c r="M12" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O12" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P12" s="21"/>
       <c r="Q12" s="45"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="31" t="s">
         <v>21</v>
       </c>
@@ -1480,40 +1480,40 @@
         <v>11</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E13" s="31"/>
       <c r="F13" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
       <c r="K13" s="21"/>
       <c r="L13" s="21"/>
       <c r="M13" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O13" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P13" s="21" t="s">
         <v>29</v>
       </c>
       <c r="Q13" s="45"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
         <v>6</v>
       </c>
@@ -1521,42 +1521,42 @@
         <v>12</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14" s="17" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="24"/>
       <c r="F14" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J14" s="21"/>
       <c r="K14" s="31"/>
       <c r="L14" s="21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="O14" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P14" s="21"/>
       <c r="Q14" s="46"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>7</v>
       </c>
@@ -1564,37 +1564,37 @@
         <v>13</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E15" s="24"/>
       <c r="F15" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I15" s="21"/>
       <c r="J15" s="21"/>
       <c r="K15" s="21"/>
       <c r="L15" s="21"/>
       <c r="M15" s="16" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N15" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="O15" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P15" s="21"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>8</v>
       </c>
@@ -1602,20 +1602,20 @@
         <v>14</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E16" s="24"/>
       <c r="F16" s="16" t="s">
         <v>28</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I16" s="21"/>
       <c r="J16" s="21"/>
@@ -1623,14 +1623,14 @@
       <c r="L16" s="21"/>
       <c r="M16" s="16"/>
       <c r="N16" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="O16" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="O16" s="16" t="s">
-        <v>138</v>
-      </c>
       <c r="P16" s="21"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="23" t="s">
         <v>9</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D17" s="19"/>
       <c r="E17" s="23"/>
@@ -1654,11 +1654,11 @@
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
       <c r="O17" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P17" s="23"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
         <v>10</v>
       </c>
@@ -1666,12 +1666,12 @@
         <v>16</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D18" s="19"/>
       <c r="E18" s="23"/>
       <c r="F18" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G18" s="18"/>
       <c r="H18" s="18"/>
@@ -1682,11 +1682,11 @@
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
       <c r="O18" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P18" s="23"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
         <v>5</v>
       </c>
@@ -1694,20 +1694,20 @@
         <v>17</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>10</v>
       </c>
       <c r="E19" s="24"/>
       <c r="F19" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
@@ -1715,15 +1715,15 @@
       <c r="L19" s="21"/>
       <c r="M19" s="16"/>
       <c r="N19" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O19" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P19" s="21"/>
       <c r="Q19" s="27"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
         <v>11</v>
       </c>
@@ -1731,40 +1731,40 @@
         <v>18</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E20" s="24"/>
       <c r="F20" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
       <c r="K20" s="31"/>
       <c r="L20" s="21"/>
       <c r="M20" s="32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N20" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O20" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P20" s="21" t="s">
         <v>29</v>
       </c>
       <c r="Q20" s="45"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" s="34" t="s">
         <v>6</v>
       </c>
@@ -1772,42 +1772,42 @@
         <v>19</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="24"/>
       <c r="F21" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I21" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J21" s="21"/>
       <c r="K21" s="31"/>
       <c r="L21" s="21"/>
       <c r="M21" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N21" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O21" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P21" s="21" t="s">
         <v>29</v>
       </c>
       <c r="Q21" s="45"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" s="35" t="s">
         <v>7</v>
       </c>
@@ -1815,20 +1815,20 @@
         <v>20</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E22" s="24"/>
       <c r="F22" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I22" s="21"/>
       <c r="J22" s="21" t="s">
@@ -1837,17 +1837,17 @@
       <c r="K22" s="31"/>
       <c r="L22" s="21"/>
       <c r="M22" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N22" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O22" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P22" s="21"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" s="34" t="s">
         <v>8</v>
       </c>
@@ -1855,37 +1855,37 @@
         <v>21</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E23" s="24"/>
       <c r="F23" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I23" s="21"/>
       <c r="J23" s="21"/>
       <c r="K23" s="31"/>
       <c r="L23" s="21"/>
       <c r="M23" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N23" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O23" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P23" s="21"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" s="36" t="s">
         <v>9</v>
       </c>
@@ -1893,12 +1893,12 @@
         <v>22</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D24" s="19"/>
       <c r="E24" s="23"/>
       <c r="F24" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
@@ -1907,15 +1907,15 @@
       <c r="K24" s="30"/>
       <c r="L24" s="23"/>
       <c r="M24" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N24" s="18"/>
       <c r="O24" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P24" s="23"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" s="36" t="s">
         <v>10</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D25" s="19"/>
       <c r="E25" s="23"/>
@@ -1937,15 +1937,15 @@
       <c r="K25" s="23"/>
       <c r="L25" s="23"/>
       <c r="M25" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N25" s="18"/>
       <c r="O25" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P25" s="23"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
         <v>5</v>
       </c>
@@ -1953,20 +1953,20 @@
         <v>24</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E26" s="24"/>
       <c r="F26" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I26" s="21"/>
       <c r="J26" s="21"/>
@@ -1974,7 +1974,7 @@
       <c r="L26" s="21"/>
       <c r="M26" s="16"/>
       <c r="N26" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O26" s="16" t="s">
         <v>26</v>
@@ -1982,7 +1982,7 @@
       <c r="P26" s="21"/>
       <c r="Q26" s="20"/>
     </row>
-    <row r="27" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="21" t="s">
         <v>21</v>
       </c>
@@ -1990,20 +1990,20 @@
         <v>25</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E27" s="21"/>
       <c r="F27" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H27" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="21"/>
@@ -2012,17 +2012,17 @@
         <v>20</v>
       </c>
       <c r="M27" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="N27" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="N27" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="O27" s="16" t="s">
         <v>26</v>
       </c>
       <c r="P27" s="21"/>
     </row>
-    <row r="28" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
         <v>6</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>26</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D28" s="17" t="s">
         <v>10</v>
@@ -2040,27 +2040,27 @@
         <v>27</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H28" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I28" s="21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J28" s="21"/>
       <c r="K28" s="31"/>
       <c r="L28" s="21"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O28" s="16" t="s">
         <v>26</v>
       </c>
       <c r="P28" s="21"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" s="21" t="s">
         <v>7</v>
       </c>
@@ -2068,20 +2068,20 @@
         <v>27</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E29" s="24"/>
       <c r="F29" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I29" s="21"/>
       <c r="J29" s="21"/>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="M29" s="21"/>
       <c r="N29" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O29" s="21" t="s">
         <v>26</v>
@@ -2100,7 +2100,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
         <v>8</v>
       </c>
@@ -2108,41 +2108,41 @@
         <v>28</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E30" s="40"/>
       <c r="F30" s="21" t="s">
         <v>31</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H30" s="21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I30" s="21"/>
       <c r="J30" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K30" s="31"/>
       <c r="L30" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M30" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N30" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O30" s="21" t="s">
         <v>26</v>
       </c>
       <c r="P30" s="21"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>9</v>
       </c>
@@ -2150,12 +2150,12 @@
         <v>29</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D31" s="19"/>
       <c r="E31" s="30"/>
       <c r="F31" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
@@ -2172,7 +2172,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" s="41" t="s">
         <v>10</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D32" s="42"/>
       <c r="E32" s="43"/>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="P32" s="41"/>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" s="21" t="s">
         <v>5</v>
       </c>
@@ -2208,20 +2208,20 @@
         <v>31</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E33" s="16"/>
       <c r="F33" s="16" t="s">
         <v>28</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H33" s="21" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I33" s="21"/>
       <c r="J33" s="31"/>
@@ -2229,7 +2229,7 @@
       <c r="L33" s="21"/>
       <c r="M33" s="16"/>
       <c r="N33" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O33" s="21" t="s">
         <v>26</v>
@@ -2237,7 +2237,7 @@
       <c r="P33" s="40"/>
       <c r="Q33" s="27"/>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -2252,11 +2252,11 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O34" s="20"/>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="5"/>
       <c r="C35" s="3"/>
@@ -2270,11 +2270,11 @@
       <c r="K35" s="9"/>
       <c r="L35" s="2"/>
       <c r="M35" s="20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P35" s="2"/>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="5" t="s">
         <v>19</v>
@@ -2287,89 +2287,89 @@
       <c r="J36" s="3"/>
       <c r="L36" s="4"/>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="5"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B38" s="5"/>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B39" s="5"/>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B40" s="33"/>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B41" s="33"/>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B42" s="33"/>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B43" s="33"/>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B44" s="5"/>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B45" s="5"/>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B46" s="5"/>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B47" s="5"/>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B48" s="5"/>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="5"/>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="5"/>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="5"/>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="5"/>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B53" s="5"/>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B54" s="5"/>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B55" s="5"/>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B56" s="5"/>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" s="5"/>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B58" s="5"/>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B59" s="5"/>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B60" s="2"/>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B61" s="2"/>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B62" s="2"/>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B63" s="2"/>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B64" s="2"/>
     </row>
   </sheetData>
@@ -2383,7 +2383,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FB24D38-8266-4755-A27E-18E23A1F5CE0}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>

</xml_diff>